<commit_message>
Replace templates with v1 (ETECOM 2026) evidence record
- Populate search log, full-text screening, codebook, coding evidence
  (84 cells), coverage matrix, gap taxonomy, PRISMA counts and the
  included-studies CSV/BibTeX with the actual v1 data; no values invented
- Keep the original coding workbook unmodified in 03_coding/source/
- Record ETECOM Table III/IV coverage and evidence next to the v1 ratings;
  mark the three re-rated NIST SP 800-210 cells (EV-012, EV-054, EV-068)
- Move the raw search exports to 01_search/exports/
- Add docs/known_issues.md, 03_coding/audit_v1_flags.csv and
  08_analysis/scripts/check_consistency.py (all checks pass)
- Fix CSA Security Guidance v5 to 2024 (key csa2024)
- Stop tracking publisher PDFs; keep only the CC BY 4.0 IEEE Access papers
- Rewrite READMEs and docs to describe the actual state of the record
</commit_message>
<xml_diff>
--- a/01_search/search_history.xlsx
+++ b/01_search/search_history.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Search History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search_History" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,21 +27,14 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -56,10 +49,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -426,17 +422,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="21.6" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="20.7" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="15.3" customWidth="1" min="6" max="6"/>
+    <col width="11.7" customWidth="1" min="7" max="7"/>
+    <col width="17.1" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -457,111 +455,325 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>fields</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>date_run</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>date_range_covered</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>date_range_filter</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>hits_returned</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>after_deduplication</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>run_by</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SRCH-0001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>EBSCOhost</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>("multi-cloud" OR "multicloud") AND ("governance" OR "compliance")</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2010-01-01 to 2025-12-31</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>TEMPLATE 000</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>TEMPLATE Initials</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>TEMPLATE row - replace with actual search run log</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SRCH-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Xplore</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>("multi-cloud" OR "multi cloud" OR "multicloud") AND ("governance" OR "security framework" OR "policy enforcement" OR "shared responsibility" OR "risk posture" OR "IAM" OR "identity federation") AND ("cloud security" OR "cybersecurity" OR "information security")</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Title/Abstract/Keywords</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2020-2025</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>SRCH-0002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>EBSCOhost</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>("hybrid cloud") AND ("policy management" OR "access control")</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-01-15</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2010-01-01 to 2025-12-31</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>EXAMPLE 000</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>EXAMPLE Initials</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EXAMPLE row - replace with actual search run log</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SRCH-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>ACM Digital Library</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>("multi-cloud" OR "multi cloud" OR "multicloud") AND ("governance" OR "security framework" OR "policy enforcement" OR "shared responsibility" OR "risk posture" OR "IAM" OR "identity federation") AND ("cloud security" OR "cybersecurity" OR "information security")</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Title/Abstract/Keywords</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2020-2025</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SRCH-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SpringerLink</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>("multi-cloud" OR "multi cloud" OR "multicloud") AND ("governance" OR "security framework" OR "policy enforcement" OR "shared responsibility" OR "risk posture" OR "IAM" OR "identity federation") AND ("cloud security" OR "cybersecurity" OR "information security")</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Title/Abstract/Keywords</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2020-2025</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>423</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>423</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SRCH-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ScienceDirect (Elsevier)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>multi-cloud AND (governance OR "security framework" OR "policy enforcement" OR "shared responsibility" OR "risk posture" OR IAM OR "identity federation") AND (cybersecurity OR "cloud security" OR "information security")</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Title/Abstract/Keywords</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>2020-2025</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>217</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>217</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Adapted syntax for ScienceDirect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SRCH-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EBSCO HOST</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>("multi-cloud" OR "multi cloud" OR "multicloud") AND ("governance" OR "security framework" OR "policy enforcement" OR "shared responsibility" OR "risk posture" OR "IAM" OR "identity federation") AND ("cloud security" OR "cybersecurity" OR "information security")</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Title/Abstract/Keywords</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>2020-2025</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>996</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>777</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Archived export (01_search/exports, sheet EBSCO) holds 777 records after EBSCO-internal deduplication; the raw 996-record export was not archived. 73 archived records carry 2026 publication dates (outside the 2020-2025 filter). EBSCO indexes IEEE Xplore (edseee) and other publisher content, so overlap with the other exports exists (docs/known_issues.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SRCH-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Citation Tracking</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Forward/backward citation tracking on Diningrat et al. (2025), Aljarrah et al. (2024), Alouffi et al. (2021): 3 records, 2 included, 1 excluded (not peer-reviewed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="n">
+        <v>1818</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>1599</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>219 duplicates removed</t>
         </is>
       </c>
     </row>

</xml_diff>